<commit_message>
Fichas V3: encabezado/pie institucional, separacion fecha/rezago, IGAE nombre oficial, INPC en puntos porcentuales, PIB en billones, redaccion prudente, tabla EMIM y ajustes visuales
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/downloads/Indicadores_Macroeconomicos_Mexico_Actualizado.xlsx
+++ b/downloads/Indicadores_Macroeconomicos_Mexico_Actualizado.xlsx
@@ -10253,7 +10253,7 @@
     <row r="2">
       <c r="A2" s="62" t="inlineStr">
         <is>
-          <t>Generado: 20/07/2026 15:14 UTC</t>
+          <t>Generado: 27/07/2026 15:52 UTC</t>
         </is>
       </c>
     </row>
@@ -10363,7 +10363,7 @@
     <row r="7">
       <c r="A7" s="64" t="inlineStr">
         <is>
-          <t>Indicador Global de Actividad Económica (IGAE)</t>
+          <t>Indicador Global de la Actividad Económica</t>
         </is>
       </c>
       <c r="B7" s="64" t="inlineStr">
@@ -11905,7 +11905,7 @@
     <row r="6">
       <c r="A6" s="82" t="inlineStr">
         <is>
-          <t>Indicador Global de Actividad Económica (IGAE)</t>
+          <t>Indicador Global de la Actividad Económica</t>
         </is>
       </c>
       <c r="B6" s="82" t="inlineStr">
@@ -12484,7 +12484,7 @@
     <row r="2">
       <c r="A2" s="62" t="inlineStr">
         <is>
-          <t>Última corrida del pipeline: 2026-07-20T15:14:35+00:00 · resultado: OK · modo: offline</t>
+          <t>Última corrida del pipeline: 2026-07-27T15:52:06+00:00 · resultado: OK · modo: offline</t>
         </is>
       </c>
     </row>
@@ -12699,7 +12699,7 @@
     <row r="7">
       <c r="A7" s="83" t="inlineStr">
         <is>
-          <t>Indicador Global de Actividad Económica (IGAE)</t>
+          <t>Indicador Global de la Actividad Económica</t>
         </is>
       </c>
       <c r="B7" s="83" t="inlineStr">

</xml_diff>

<commit_message>
Conexión de indicadores INEGI restantes (feature/conexion-inegi-restantes).
- Confirma y conecta PIB (737372, 737375), IGAE (737121), IMAI (737233, 737234),
  Balanza comercial (33223, 33226), Tasa de desocupación (444603) e INPC
  (334360, 334452) vía API oficial del INEGI (BIE).
- Extiende scripts/sources/inegi.py para soportar múltiples series por
  indicador, factores y transformaciones (yoy, mom, qoq, diff_yoy_pp).
- Actualiza build_data.py para fusionar series INEGI sobre sus columnas
  objetivo sin borrar columnas de respaldo.
- Registra PIBSEC, Consumo, IMFBCF, IOAE y EMIM como pendientes de confirmar
  serie, conservando sus datos de respaldo.
- Regenera datos, CSV, Excel y resumen con el pipeline en modo online.

Resultado: 24 passed en pytest, 0 errores críticos en validate.py.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/downloads/Indicadores_Macroeconomicos_Mexico_Actualizado.xlsx
+++ b/downloads/Indicadores_Macroeconomicos_Mexico_Actualizado.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18465" tabRatio="600" firstSheet="1" activeTab="6" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Síntesis de coyuntura" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="PIB" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="PIB Sectorial" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="IGAE" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="IMAI" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Exportaciones" sheetId="6" state="hidden" r:id="rId6"/>
-    <sheet name="Balanza comercial" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Consumo Privado" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="IED" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Tasa de desocupación" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="INPC (Inflación)" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Formación bruta capital fijo" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="IOAE" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="EMIM (Manufactura)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Metodología y fuentes" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Control de actualizaciones" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Síntesis de coyuntura" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIB Sectorial" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IGAE" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IMAI" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exportaciones" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balanza comercial" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumo Privado" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IED" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasa de desocupación" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INPC (Inflación)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formación bruta capital fijo" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IOAE" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EMIM (Manufactura)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metodología y fuentes" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control de actualizaciones" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -832,14 +832,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1800" b="1" i="0" strike="noStrike" kern="1200" spc="0" normalizeH="0" baseline="0">
                 <a:solidFill>
@@ -882,16 +882,16 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1800" b="1" i="0" strike="noStrike" kern="1200" spc="0" normalizeH="0" baseline="0">
               <a:solidFill>
@@ -933,10 +933,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="1E5B4F"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -959,18 +959,18 @@
               <idx val="18"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="800" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -1000,7 +1000,7 @@
           </dLbls>
           <trendline>
             <spPr>
-              <a:ln w="19050" cap="rnd">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050" cap="rnd">
                 <a:solidFill>
                   <a:schemeClr val="accent1"/>
                 </a:solidFill>
@@ -1187,7 +1187,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="38100" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="38100" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="A6802D"/>
               </a:solidFill>
@@ -1198,7 +1198,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1235,23 +1235,23 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:sysClr val="windowText" lastClr="000000">
                   <a:lumOff val="85000"/>
                   <a:lumMod val="15000"/>
                 </a:sysClr>
               </a:solidFill>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -1449,8 +1449,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -1462,9 +1462,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" spc="0" normalizeH="0" baseline="0">
                 <a:solidFill>
@@ -1500,7 +1500,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="15000"/>
@@ -1514,7 +1514,7 @@
         </majorGridlines>
         <minorGridlines>
           <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="5000"/>
@@ -1529,9 +1529,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" cap="all" baseline="0">
                     <a:solidFill>
@@ -1554,16 +1554,16 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill/>
-            <a:ln>
+            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:pPr>
                 <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" cap="all" baseline="0">
                   <a:solidFill>
@@ -1588,16 +1588,16 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -1650,16 +1650,16 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -1688,16 +1688,16 @@
       <legendPos val="t"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -1722,10 +1722,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
           <a:lumMod val="15000"/>
@@ -1740,14 +1740,14 @@
 </file>
 
 <file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -1770,16 +1770,16 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -1820,7 +1820,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28575" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="1E5B4F"/>
               </a:solidFill>
@@ -1832,10 +1832,10 @@
             <symbol val="circle"/>
             <size val="5"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="1E5B4F"/>
               </a:solidFill>
-              <a:ln w="9525">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
                 <a:solidFill>
                   <a:srgbClr val="1E5B4F"/>
                 </a:solidFill>
@@ -1847,10 +1847,10 @@
             <dLbl>
               <idx val="9"/>
               <spPr>
-                <a:solidFill>
+                <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:sysClr val="window" lastClr="FFFFFF"/>
                 </a:solidFill>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:solidFill>
                     <a:sysClr val="windowText" lastClr="000000">
                       <a:lumOff val="75000"/>
@@ -1861,11 +1861,11 @@
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:spAutoFit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -1904,18 +1904,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -2047,7 +2047,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28575" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="9C2348"/>
               </a:solidFill>
@@ -2059,10 +2059,10 @@
             <symbol val="circle"/>
             <size val="5"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9C2348"/>
               </a:solidFill>
-              <a:ln w="9525">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
                 <a:solidFill>
                   <a:srgbClr val="9C2348"/>
                 </a:solidFill>
@@ -2081,18 +2081,18 @@
               <idx val="10"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -2224,7 +2224,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28575" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="A6802D"/>
               </a:solidFill>
@@ -2236,10 +2236,10 @@
             <symbol val="circle"/>
             <size val="5"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="A6802D"/>
               </a:solidFill>
-              <a:ln w="9525">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
                 <a:solidFill>
                   <a:srgbClr val="A6802D"/>
                 </a:solidFill>
@@ -2271,18 +2271,18 @@
             <dLbl>
               <idx val="10"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:spAutoFit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="900" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -2318,18 +2318,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -2461,7 +2461,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28575" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="0070C0"/>
               </a:solidFill>
@@ -2473,10 +2473,10 @@
             <symbol val="circle"/>
             <size val="5"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="0070C0"/>
               </a:solidFill>
-              <a:ln w="9525">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
                 <a:solidFill>
                   <a:srgbClr val="0070C0"/>
                 </a:solidFill>
@@ -2496,18 +2496,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -2650,8 +2650,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -2663,9 +2663,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -2703,7 +2703,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="15000"/>
@@ -2720,16 +2720,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -2758,16 +2758,16 @@
       <legendPos val="t"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -2792,10 +2792,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
           <a:lumMod val="15000"/>
@@ -2810,14 +2810,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1400" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -2845,16 +2845,16 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1400" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -2896,10 +2896,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="002F2A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -3016,10 +3016,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="1E5B4F"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -3136,10 +3136,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="9C2348"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -3147,18 +3147,18 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -3312,7 +3312,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28575" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="A6802D"/>
               </a:solidFill>
@@ -3324,10 +3324,10 @@
             <symbol val="circle"/>
             <size val="5"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="A6802D"/>
               </a:solidFill>
-              <a:ln w="9525">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
                 <a:solidFill>
                   <a:srgbClr val="A6802D"/>
                 </a:solidFill>
@@ -3337,18 +3337,18 @@
           </marker>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -3472,8 +3472,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -3485,9 +3485,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -3524,7 +3524,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="15000"/>
@@ -3539,9 +3539,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -3564,16 +3564,16 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill/>
-            <a:ln>
+            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:pPr>
                 <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
@@ -3599,16 +3599,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -3661,16 +3661,16 @@
         <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -3699,16 +3699,16 @@
       <legendPos val="t"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -3733,10 +3733,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
           <a:lumMod val="15000"/>
@@ -3751,14 +3751,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -3781,16 +3781,16 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -3831,7 +3831,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="38100" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="38100" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="1E5B4F"/>
               </a:solidFill>
@@ -3843,10 +3843,10 @@
             <symbol val="circle"/>
             <size val="5"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="1E5B4F"/>
               </a:solidFill>
-              <a:ln w="19050">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
                 <a:solidFill>
                   <a:srgbClr val="1E5B4F"/>
                 </a:solidFill>
@@ -3871,18 +3871,18 @@
             <dLbl>
               <idx val="11"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:spAutoFit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="900" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -3907,18 +3907,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -3949,7 +3949,7 @@
           </dLbls>
           <trendline>
             <spPr>
-              <a:ln w="19050" cap="rnd">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050" cap="rnd">
                 <a:solidFill>
                   <a:schemeClr val="accent1"/>
                 </a:solidFill>
@@ -4066,7 +4066,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28575" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="A6802D"/>
               </a:solidFill>
@@ -4077,7 +4077,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -4094,18 +4094,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -4240,7 +4240,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28575" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="9C2348"/>
               </a:solidFill>
@@ -4252,10 +4252,10 @@
             <symbol val="circle"/>
             <size val="5"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9C2348"/>
               </a:solidFill>
-              <a:ln w="9525">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
                 <a:solidFill>
                   <a:srgbClr val="9C2348"/>
                 </a:solidFill>
@@ -4281,18 +4281,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -4437,8 +4437,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -4450,9 +4450,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -4489,7 +4489,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="15000"/>
@@ -4506,16 +4506,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -4544,16 +4544,16 @@
       <legendPos val="t"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -4578,10 +4578,10 @@
     <dispBlanksAs val="zero"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
           <a:lumMod val="15000"/>
@@ -4596,14 +4596,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -4634,16 +4634,16 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -4685,10 +4685,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="1E5B4F"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -4699,10 +4699,10 @@
             <invertIfNegative val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9C2348"/>
               </a:solidFill>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -4712,16 +4712,16 @@
             <dLbl>
               <idx val="9"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="900" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -4756,16 +4756,16 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -4795,7 +4795,7 @@
           </dLbls>
           <trendline>
             <spPr>
-              <a:ln w="19050" cap="rnd">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050" cap="rnd">
                 <a:solidFill>
                   <a:schemeClr val="accent1"/>
                 </a:solidFill>
@@ -4927,7 +4927,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28575" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="A6802D"/>
               </a:solidFill>
@@ -4939,10 +4939,10 @@
             <symbol val="circle"/>
             <size val="5"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="A6802D"/>
               </a:solidFill>
-              <a:ln w="9525">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
                 <a:solidFill>
                   <a:srgbClr val="A6802D"/>
                 </a:solidFill>
@@ -4954,16 +4954,16 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -5004,10 +5004,10 @@
             <dLbl>
               <idx val="9"/>
               <spPr>
-                <a:solidFill>
+                <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:sysClr val="window" lastClr="FFFFFF"/>
                 </a:solidFill>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:solidFill>
                     <a:sysClr val="windowText" lastClr="000000">
                       <a:lumOff val="75000"/>
@@ -5018,11 +5018,11 @@
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
                   <a:spAutoFit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="900" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -5050,16 +5050,16 @@
             <dLbl>
               <idx val="10"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -5085,16 +5085,16 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -5239,8 +5239,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -5252,9 +5252,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -5290,7 +5290,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="15000"/>
@@ -5305,9 +5305,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -5330,16 +5330,16 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill/>
-            <a:ln>
+            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:pPr>
                 <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
@@ -5365,16 +5365,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -5427,16 +5427,16 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -5465,16 +5465,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -5499,10 +5499,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
           <a:lumMod val="15000"/>
@@ -5517,14 +5517,14 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -5556,16 +5556,16 @@
       <layout/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -5607,10 +5607,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="1E5B4F"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="1E5B4F"/>
               </a:solidFill>
@@ -5817,7 +5817,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="38100" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="38100" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="A6802D"/>
               </a:solidFill>
@@ -5828,7 +5828,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -5895,18 +5895,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -6087,8 +6087,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -6100,9 +6100,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -6138,7 +6138,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="15000"/>
@@ -6155,16 +6155,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -6217,16 +6217,16 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -6256,16 +6256,16 @@
       <layout/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -6290,10 +6290,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
           <a:lumMod val="15000"/>
@@ -6308,14 +6308,14 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1400" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -6339,16 +6339,16 @@
       <layout/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1400" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -6390,10 +6390,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="9C2348"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -6403,18 +6403,18 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:spAutoFit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="900" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -6442,18 +6442,18 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:spAutoFit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="900" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -6481,18 +6481,18 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:spAutoFit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="900" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -6520,18 +6520,18 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:spAutoFit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="900" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -6559,18 +6559,18 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:spAutoFit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="900" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -6596,18 +6596,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -6638,7 +6638,7 @@
           </dLbls>
           <trendline>
             <spPr>
-              <a:ln w="19050" cap="rnd">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050" cap="rnd">
                 <a:solidFill>
                   <a:schemeClr val="accent1"/>
                 </a:solidFill>
@@ -6832,10 +6832,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="1E5B4F"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -7034,8 +7034,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -7047,9 +7047,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -7085,7 +7085,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="15000"/>
@@ -7100,9 +7100,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -7131,16 +7131,16 @@
           <layout/>
           <overlay val="0"/>
           <spPr>
-            <a:noFill/>
-            <a:ln>
+            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:pPr>
                 <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
@@ -7166,16 +7166,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -7205,16 +7205,16 @@
       <layout/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -7239,10 +7239,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
           <a:lumMod val="15000"/>
@@ -7257,14 +7257,14 @@
 </file>
 
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -7287,16 +7287,16 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -7337,7 +7337,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:pattFill prst="pct20">
+            <a:pattFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="pct20">
               <a:fgClr>
                 <a:srgbClr val="1E5B4F"/>
               </a:fgClr>
@@ -7345,7 +7345,7 @@
                 <a:schemeClr val="bg1"/>
               </a:bgClr>
             </a:pattFill>
-            <a:ln w="38100">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="38100">
               <a:solidFill>
                 <a:srgbClr val="1E5B4F"/>
               </a:solidFill>
@@ -7354,16 +7354,16 @@
           </spPr>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -7510,7 +7510,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28575" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="A6802D"/>
               </a:solidFill>
@@ -7522,10 +7522,10 @@
             <symbol val="circle"/>
             <size val="5"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="A6802D"/>
               </a:solidFill>
-              <a:ln w="9525">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
                 <a:solidFill>
                   <a:srgbClr val="A6802D"/>
                 </a:solidFill>
@@ -7585,16 +7585,16 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -7772,16 +7772,16 @@
         <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -7810,16 +7810,16 @@
       <legendPos val="t"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -7844,10 +7844,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
           <a:lumMod val="15000"/>
@@ -7862,14 +7862,14 @@
 </file>
 
 <file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -7897,16 +7897,16 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -7948,10 +7948,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="002F2A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -8116,10 +8116,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="1E5B4F"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -8284,10 +8284,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="9C2348"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -8468,7 +8468,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28575" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="A6802D"/>
               </a:solidFill>
@@ -8480,10 +8480,10 @@
             <symbol val="circle"/>
             <size val="5"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="A6802D"/>
               </a:solidFill>
-              <a:ln w="9525">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
                 <a:solidFill>
                   <a:srgbClr val="A6802D"/>
                 </a:solidFill>
@@ -8496,18 +8496,18 @@
               <idx val="18"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -8706,8 +8706,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -8719,9 +8719,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="800" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -8757,7 +8757,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="15000"/>
@@ -8774,16 +8774,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="800" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -8812,16 +8812,16 @@
       <legendPos val="t"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -8846,10 +8846,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
           <a:lumMod val="15000"/>
@@ -8864,14 +8864,14 @@
 </file>
 
 <file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -8894,16 +8894,16 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -8944,7 +8944,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28575" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="1E5B4F"/>
               </a:solidFill>
@@ -8956,10 +8956,10 @@
             <symbol val="circle"/>
             <size val="5"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="1E5B4F"/>
               </a:solidFill>
-              <a:ln w="9525">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
                 <a:solidFill>
                   <a:srgbClr val="1E5B4F"/>
                 </a:solidFill>
@@ -9011,16 +9011,16 @@
             <dLbl>
               <idx val="9"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="900" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -9059,16 +9059,16 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -9219,7 +9219,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28575" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="0070C0"/>
               </a:solidFill>
@@ -9230,7 +9230,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -9257,16 +9257,16 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -9410,8 +9410,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -9423,9 +9423,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -9462,7 +9462,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="15000"/>
@@ -9478,16 +9478,16 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -9542,16 +9542,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -9580,16 +9580,16 @@
       <legendPos val="t"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -9614,10 +9614,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
           <a:lumMod val="15000"/>
@@ -9632,7 +9632,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>5</col>
@@ -9652,9 +9652,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -9664,7 +9664,7 @@
 </file>
 
 <file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>7</col>
@@ -9684,9 +9684,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -9696,7 +9696,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>7</col>
@@ -9716,9 +9716,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -9728,7 +9728,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>6</col>
@@ -9748,9 +9748,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -9760,7 +9760,7 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>5</col>
@@ -9780,9 +9780,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -9792,7 +9792,7 @@
 </file>
 
 <file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>4</col>
@@ -9812,9 +9812,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -9824,7 +9824,7 @@
 </file>
 
 <file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>5</col>
@@ -9844,9 +9844,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -9856,7 +9856,7 @@
 </file>
 
 <file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>5</col>
@@ -9876,9 +9876,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -9888,7 +9888,7 @@
 </file>
 
 <file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>7</col>
@@ -9908,9 +9908,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -9920,7 +9920,7 @@
 </file>
 
 <file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>5</col>
@@ -9940,9 +9940,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -10253,7 +10253,7 @@
     <row r="2">
       <c r="A2" s="62" t="inlineStr">
         <is>
-          <t>Generado: 31/07/2026 15:13 UTC</t>
+          <t>Generado: 03/08/2026 03:31 UTC</t>
         </is>
       </c>
     </row>
@@ -10316,10 +10316,10 @@
         </is>
       </c>
       <c r="E5" s="64" t="n">
-        <v>24973976.1</v>
+        <v>24973976.071</v>
       </c>
       <c r="F5" s="64" t="n">
-        <v>0.002423004906679571</v>
+        <v>0.002423</v>
       </c>
       <c r="G5" s="64" t="inlineStr">
         <is>
@@ -10330,7 +10330,7 @@
     <row r="6">
       <c r="A6" s="65" t="inlineStr">
         <is>
-          <t>Producto Interno Bruto por actividad económica</t>
+          <t>Producto Interno Bruto por sector de actividad</t>
         </is>
       </c>
       <c r="B6" s="65" t="inlineStr">
@@ -10394,7 +10394,7 @@
     <row r="8">
       <c r="A8" s="65" t="inlineStr">
         <is>
-          <t>Indicador Mensual de Actividad Industrial (IMAI)</t>
+          <t>Indicador Mensual de la Actividad Industrial</t>
         </is>
       </c>
       <c r="B8" s="65" t="inlineStr">
@@ -10409,14 +10409,14 @@
       </c>
       <c r="D8" s="65" t="inlineStr">
         <is>
-          <t>Abr 26 P</t>
+          <t>May 26</t>
         </is>
       </c>
       <c r="E8" s="65" t="n">
-        <v>102.4</v>
+        <v>101.629971</v>
       </c>
       <c r="F8" s="65" t="n">
-        <v>0.02093718843469605</v>
+        <v>-0.007713</v>
       </c>
       <c r="G8" s="65" t="inlineStr">
         <is>
@@ -10427,7 +10427,7 @@
     <row r="9">
       <c r="A9" s="64" t="inlineStr">
         <is>
-          <t>Balanza comercial de mercancías de México</t>
+          <t>Balanza comercial</t>
         </is>
       </c>
       <c r="B9" s="64" t="inlineStr">
@@ -10442,14 +10442,14 @@
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>May 26 O</t>
+          <t>Jun 26</t>
         </is>
       </c>
       <c r="E9" s="64" t="n">
-        <v>69544.49099999999</v>
+        <v>72551.015</v>
       </c>
       <c r="F9" s="64" t="n">
-        <v>67285.323</v>
+        <v>68461.11900000001</v>
       </c>
       <c r="G9" s="64" t="inlineStr">
         <is>
@@ -10460,7 +10460,7 @@
     <row r="10">
       <c r="A10" s="65" t="inlineStr">
         <is>
-          <t>Tasa de desocupación nacional</t>
+          <t>Tasa de desocupación</t>
         </is>
       </c>
       <c r="B10" s="65" t="inlineStr">
@@ -10475,11 +10475,11 @@
       </c>
       <c r="D10" s="65" t="inlineStr">
         <is>
-          <t>May 26</t>
+          <t>Jun 26</t>
         </is>
       </c>
       <c r="E10" s="65" t="n">
-        <v>0.027</v>
+        <v>0.028985</v>
       </c>
       <c r="F10" s="65" t="n"/>
       <c r="G10" s="65" t="inlineStr">
@@ -10491,7 +10491,7 @@
     <row r="11">
       <c r="A11" s="64" t="inlineStr">
         <is>
-          <t>Índice Nacional de Precios al Consumidor (INPC)</t>
+          <t>Índice de Precios al Consumidor</t>
         </is>
       </c>
       <c r="B11" s="64" t="inlineStr">
@@ -10506,14 +10506,14 @@
       </c>
       <c r="D11" s="64" t="inlineStr">
         <is>
-          <t>May 26</t>
+          <t>Jun 26</t>
         </is>
       </c>
       <c r="E11" s="64" t="n">
-        <v>3.94</v>
+        <v>3.365977</v>
       </c>
       <c r="F11" s="64" t="n">
-        <v>4.19</v>
+        <v>4.03192</v>
       </c>
       <c r="G11" s="64" t="inlineStr">
         <is>
@@ -10524,7 +10524,7 @@
     <row r="12">
       <c r="A12" s="65" t="inlineStr">
         <is>
-          <t>Indicador Mensual de Consumo Privado</t>
+          <t>Indicador mensual del consumo privado</t>
         </is>
       </c>
       <c r="B12" s="65" t="inlineStr">
@@ -11583,7 +11583,7 @@
     <row r="2">
       <c r="A2" s="62" t="inlineStr">
         <is>
-          <t>Fuente: INEGI · Frecuencia: Mensual · Unidad: Índice base 2018=100 · Estado: pendiente de token</t>
+          <t>Fuente: INEGI · Frecuencia: Mensual · Unidad: Índice base 2018=100 · Estado: pendiente de confirmar serie</t>
         </is>
       </c>
     </row>
@@ -11645,7 +11645,7 @@
     <row r="2">
       <c r="A2" s="62" t="inlineStr">
         <is>
-          <t>Fuente: INEGI · Frecuencia: Mensual · Unidad: Variación mensual estimada (%) · Estado: pendiente de token</t>
+          <t>Fuente: INEGI · Frecuencia: Mensual · Unidad: Variación mensual estimada (%) · Estado: pendiente de confirmar serie</t>
         </is>
       </c>
     </row>
@@ -11711,7 +11711,7 @@
     <row r="2">
       <c r="A2" s="62" t="inlineStr">
         <is>
-          <t>Fuente: INEGI · Frecuencia: Mensual · Unidad: Índice · Estado: pendiente de token</t>
+          <t>Fuente: INEGI · Frecuencia: Mensual · Unidad: Índice · Estado: pendiente de confirmar serie</t>
         </is>
       </c>
     </row>
@@ -11829,7 +11829,7 @@
       </c>
       <c r="C4" s="82" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>737375</t>
         </is>
       </c>
       <c r="D4" s="82" t="inlineStr">
@@ -11854,14 +11854,14 @@
       </c>
       <c r="H4" s="82" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/app/indicadores/?tm=3#D733671_600917</t>
+          <t>https://www.inegi.org.mx/app/indicadores/?tm=3&amp;t=605598#D737375</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="83" t="inlineStr">
         <is>
-          <t>Producto Interno Bruto por actividad económica</t>
+          <t>Producto Interno Bruto por sector de actividad</t>
         </is>
       </c>
       <c r="B5" s="83" t="inlineStr">
@@ -11938,14 +11938,14 @@
       </c>
       <c r="H6" s="82" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/app/indicadores/?tm=3&amp;t=1090#D737121</t>
+          <t>https://www.inegi.org.mx/app/indicadores/?tm=3&amp;t=603589#D737121</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="83" t="inlineStr">
         <is>
-          <t>Indicador Mensual de Actividad Industrial (IMAI)</t>
+          <t>Indicador Mensual de la Actividad Industrial</t>
         </is>
       </c>
       <c r="B7" s="83" t="inlineStr">
@@ -11955,7 +11955,7 @@
       </c>
       <c r="C7" s="83" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>737234</t>
         </is>
       </c>
       <c r="D7" s="83" t="inlineStr">
@@ -11980,14 +11980,14 @@
       </c>
       <c r="H7" s="83" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/temas/imai/</t>
+          <t>https://www.inegi.org.mx/app/indicadores/?tm=3&amp;t=603729#D737234</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="82" t="inlineStr">
         <is>
-          <t>Balanza comercial de mercancías de México</t>
+          <t>Balanza comercial</t>
         </is>
       </c>
       <c r="B8" s="82" t="inlineStr">
@@ -11997,7 +11997,7 @@
       </c>
       <c r="C8" s="82" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>33226</t>
         </is>
       </c>
       <c r="D8" s="82" t="inlineStr">
@@ -12022,14 +12022,14 @@
       </c>
       <c r="H8" s="82" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/temas/balanza/#informacion_general</t>
+          <t>https://www.inegi.org.mx/app/indicadores/?tm=3&amp;t=36695#D33226</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="83" t="inlineStr">
         <is>
-          <t>Tasa de desocupación nacional</t>
+          <t>Tasa de desocupación</t>
         </is>
       </c>
       <c r="B9" s="83" t="inlineStr">
@@ -12039,7 +12039,7 @@
       </c>
       <c r="C9" s="83" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>444603</t>
         </is>
       </c>
       <c r="D9" s="83" t="inlineStr">
@@ -12064,14 +12064,14 @@
       </c>
       <c r="H9" s="83" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/temas/empleo/</t>
+          <t>https://www.inegi.org.mx/app/indicadores/?tm=3&amp;t=4#D444603</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="82" t="inlineStr">
         <is>
-          <t>Índice Nacional de Precios al Consumidor (INPC)</t>
+          <t>Índice de Precios al Consumidor</t>
         </is>
       </c>
       <c r="B10" s="82" t="inlineStr">
@@ -12081,7 +12081,7 @@
       </c>
       <c r="C10" s="82" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>334452</t>
         </is>
       </c>
       <c r="D10" s="82" t="inlineStr">
@@ -12106,14 +12106,14 @@
       </c>
       <c r="H10" s="82" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/temas/inpc/</t>
+          <t>https://www.inegi.org.mx/app/indicadores/?tm=3&amp;t=682416#D334452</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="83" t="inlineStr">
         <is>
-          <t>Indicador Mensual de Consumo Privado</t>
+          <t>Indicador mensual del consumo privado</t>
         </is>
       </c>
       <c r="B11" s="83" t="inlineStr">
@@ -12482,7 +12482,7 @@
     <row r="2">
       <c r="A2" s="62" t="inlineStr">
         <is>
-          <t>Última corrida del pipeline: 2026-07-31T15:13:20+00:00 · resultado: OK · modo: offline</t>
+          <t>Última corrida del pipeline: 2026-08-03T03:31:44+00:00 · resultado: OK · modo: offline</t>
         </is>
       </c>
     </row>
@@ -12571,12 +12571,12 @@
       </c>
       <c r="C5" s="83" t="inlineStr">
         <is>
-          <t>dato de respaldo vigente</t>
+          <t>actualizado automáticamente</t>
         </is>
       </c>
       <c r="D5" s="83" t="inlineStr">
         <is>
-          <t>respaldo</t>
+          <t>api</t>
         </is>
       </c>
       <c r="E5" s="83" t="inlineStr">
@@ -12586,7 +12586,7 @@
       </c>
       <c r="F5" s="83" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G5" s="83" t="inlineStr">
@@ -12611,12 +12611,12 @@
       </c>
       <c r="K5" s="83" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="L5" s="83" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="M5" s="83" t="inlineStr">
@@ -12629,7 +12629,7 @@
     <row r="6">
       <c r="A6" s="82" t="inlineStr">
         <is>
-          <t>Producto Interno Bruto por actividad económica</t>
+          <t>Producto Interno Bruto por sector de actividad</t>
         </is>
       </c>
       <c r="B6" s="82" t="inlineStr">
@@ -12747,12 +12747,12 @@
       </c>
       <c r="K7" s="83" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="L7" s="83" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="M7" s="83" t="inlineStr">
@@ -12765,7 +12765,7 @@
     <row r="8">
       <c r="A8" s="84" t="inlineStr">
         <is>
-          <t>Indicador Mensual de Actividad Industrial (IMAI)</t>
+          <t>Indicador Mensual de la Actividad Industrial</t>
         </is>
       </c>
       <c r="B8" s="84" t="inlineStr">
@@ -12775,12 +12775,12 @@
       </c>
       <c r="C8" s="84" t="inlineStr">
         <is>
-          <t>dato en revisión</t>
+          <t>actualizado automáticamente</t>
         </is>
       </c>
       <c r="D8" s="84" t="inlineStr">
         <is>
-          <t>respaldo</t>
+          <t>api</t>
         </is>
       </c>
       <c r="E8" s="84" t="inlineStr">
@@ -12790,17 +12790,17 @@
       </c>
       <c r="F8" s="84" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G8" s="84" t="inlineStr">
         <is>
-          <t>Abr 26 P</t>
+          <t>May 26</t>
         </is>
       </c>
       <c r="H8" s="84" t="inlineStr">
         <is>
-          <t>Abr 26 P</t>
+          <t>May 26</t>
         </is>
       </c>
       <c r="I8" s="84" t="n"/>
@@ -12811,12 +12811,12 @@
       </c>
       <c r="K8" s="84" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="L8" s="84" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="M8" s="84" t="inlineStr">
@@ -12833,7 +12833,7 @@
     <row r="9">
       <c r="A9" s="83" t="inlineStr">
         <is>
-          <t>Balanza comercial de mercancías de México</t>
+          <t>Balanza comercial</t>
         </is>
       </c>
       <c r="B9" s="83" t="inlineStr">
@@ -12843,12 +12843,12 @@
       </c>
       <c r="C9" s="83" t="inlineStr">
         <is>
-          <t>dato de respaldo vigente</t>
+          <t>actualizado automáticamente</t>
         </is>
       </c>
       <c r="D9" s="83" t="inlineStr">
         <is>
-          <t>respaldo</t>
+          <t>api</t>
         </is>
       </c>
       <c r="E9" s="83" t="inlineStr">
@@ -12858,17 +12858,17 @@
       </c>
       <c r="F9" s="83" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G9" s="83" t="inlineStr">
         <is>
-          <t>May 26 O</t>
+          <t>Jun 26</t>
         </is>
       </c>
       <c r="H9" s="83" t="inlineStr">
         <is>
-          <t>May 26 O</t>
+          <t>Jun 26</t>
         </is>
       </c>
       <c r="I9" s="83" t="inlineStr">
@@ -12883,12 +12883,12 @@
       </c>
       <c r="K9" s="83" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="L9" s="83" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="M9" s="83" t="inlineStr">
@@ -12901,7 +12901,7 @@
     <row r="10">
       <c r="A10" s="82" t="inlineStr">
         <is>
-          <t>Tasa de desocupación nacional</t>
+          <t>Tasa de desocupación</t>
         </is>
       </c>
       <c r="B10" s="82" t="inlineStr">
@@ -12911,12 +12911,12 @@
       </c>
       <c r="C10" s="82" t="inlineStr">
         <is>
-          <t>dato de respaldo vigente</t>
+          <t>actualizado automáticamente</t>
         </is>
       </c>
       <c r="D10" s="82" t="inlineStr">
         <is>
-          <t>respaldo</t>
+          <t>api</t>
         </is>
       </c>
       <c r="E10" s="82" t="inlineStr">
@@ -12926,17 +12926,17 @@
       </c>
       <c r="F10" s="82" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G10" s="82" t="inlineStr">
         <is>
-          <t>May 26</t>
+          <t>Jun 26</t>
         </is>
       </c>
       <c r="H10" s="82" t="inlineStr">
         <is>
-          <t>May 26</t>
+          <t>Jun 26</t>
         </is>
       </c>
       <c r="I10" s="82" t="inlineStr">
@@ -12951,12 +12951,12 @@
       </c>
       <c r="K10" s="82" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="L10" s="82" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="M10" s="82" t="inlineStr">
@@ -12969,7 +12969,7 @@
     <row r="11">
       <c r="A11" s="83" t="inlineStr">
         <is>
-          <t>Índice Nacional de Precios al Consumidor (INPC)</t>
+          <t>Índice de Precios al Consumidor</t>
         </is>
       </c>
       <c r="B11" s="83" t="inlineStr">
@@ -12979,12 +12979,12 @@
       </c>
       <c r="C11" s="83" t="inlineStr">
         <is>
-          <t>dato de respaldo vigente</t>
+          <t>actualizado automáticamente</t>
         </is>
       </c>
       <c r="D11" s="83" t="inlineStr">
         <is>
-          <t>respaldo</t>
+          <t>api</t>
         </is>
       </c>
       <c r="E11" s="83" t="inlineStr">
@@ -12994,17 +12994,17 @@
       </c>
       <c r="F11" s="83" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G11" s="83" t="inlineStr">
         <is>
-          <t>May 26</t>
+          <t>Jun 26</t>
         </is>
       </c>
       <c r="H11" s="83" t="inlineStr">
         <is>
-          <t>May 26</t>
+          <t>Jun 26</t>
         </is>
       </c>
       <c r="I11" s="83" t="n"/>
@@ -13015,12 +13015,12 @@
       </c>
       <c r="K11" s="83" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="L11" s="83" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="M11" s="83" t="inlineStr">
@@ -13033,7 +13033,7 @@
     <row r="12">
       <c r="A12" s="84" t="inlineStr">
         <is>
-          <t>Indicador Mensual de Consumo Privado</t>
+          <t>Indicador mensual del consumo privado</t>
         </is>
       </c>
       <c r="B12" s="84" t="inlineStr">
@@ -13115,7 +13115,7 @@
       </c>
       <c r="C13" s="83" t="inlineStr">
         <is>
-          <t>pendiente de token</t>
+          <t>pendiente de confirmar serie</t>
         </is>
       </c>
       <c r="D13" s="83" t="inlineStr">
@@ -13167,7 +13167,7 @@
       </c>
       <c r="C14" s="82" t="inlineStr">
         <is>
-          <t>pendiente de token</t>
+          <t>pendiente de confirmar serie</t>
         </is>
       </c>
       <c r="D14" s="82" t="inlineStr">
@@ -13219,7 +13219,7 @@
       </c>
       <c r="C15" s="83" t="inlineStr">
         <is>
-          <t>pendiente de token</t>
+          <t>pendiente de confirmar serie</t>
         </is>
       </c>
       <c r="D15" s="83" t="inlineStr">
@@ -13492,21 +13492,21 @@
     <row r="23">
       <c r="A23" s="62" t="inlineStr">
         <is>
-          <t>• [IMFBCF] sin observaciones (estado: pendiente de token).</t>
+          <t>• [IMFBCF] sin observaciones (estado: pendiente de confirmar serie).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="62" t="inlineStr">
         <is>
-          <t>• [IOAE] sin observaciones (estado: pendiente de token).</t>
+          <t>• [IOAE] sin observaciones (estado: pendiente de confirmar serie).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="62" t="inlineStr">
         <is>
-          <t>• [EMIM] sin observaciones (estado: pendiente de token).</t>
+          <t>• [EMIM] sin observaciones (estado: pendiente de confirmar serie).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): re-genera datos y Excel en modo online tras validación.
- Actualiza data/indicadores.json, manifest, summary, update_log y Excel
  con el pipeline online usando INEGI_TOKEN.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/downloads/Indicadores_Macroeconomicos_Mexico_Actualizado.xlsx
+++ b/downloads/Indicadores_Macroeconomicos_Mexico_Actualizado.xlsx
@@ -10253,7 +10253,7 @@
     <row r="2">
       <c r="A2" s="62" t="inlineStr">
         <is>
-          <t>Generado: 03/08/2026 03:31 UTC</t>
+          <t>Generado: 03/08/2026 04:28 UTC</t>
         </is>
       </c>
     </row>
@@ -12453,7 +12453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -12482,7 +12482,7 @@
     <row r="2">
       <c r="A2" s="62" t="inlineStr">
         <is>
-          <t>Última corrida del pipeline: 2026-08-03T03:31:44+00:00 · resultado: OK · modo: offline</t>
+          <t>Última corrida del pipeline: 2026-08-03T04:28:50+00:00 · resultado: OK · modo: online</t>
         </is>
       </c>
     </row>
@@ -13492,40 +13492,117 @@
     <row r="23">
       <c r="A23" s="62" t="inlineStr">
         <is>
-          <t>• [IMFBCF] sin observaciones (estado: pendiente de confirmar serie).</t>
+          <t>• BANXICO_TOKEN ausente: se omiten tipo de cambio y tasa objetivo; se conservan datos previos.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="62" t="inlineStr">
         <is>
-          <t>• [IOAE] sin observaciones (estado: pendiente de confirmar serie).</t>
+          <t>• INEGI PIB: 33 observaciones (serie 737372, base BIE-BISE); última 1T-26 = 24973976.071; actualización BIE 18/06/2026 12:00:00 a. m..</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="62" t="inlineStr">
         <is>
-          <t>• [EMIM] sin observaciones (estado: pendiente de confirmar serie).</t>
+          <t>• INEGI PIB: 33 observaciones (serie 737375, base BIE-BISE); última 1T-26 = 0.002423; actualización BIE 18/06/2026 12:00:00 a. m..</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="62" t="inlineStr">
         <is>
-          <t>• [TIPOCAMBIO] sin observaciones (estado: pendiente de token).</t>
+          <t>• INEGI IGAE: 101 observaciones (serie 737121, base BIE-BISE); última May 26 = 108.595752; actualización BIE 23/07/2026 12:00:00 a. m..</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="62" t="inlineStr">
         <is>
-          <t>• [TASA] sin observaciones (estado: pendiente de token).</t>
+          <t>• INEGI IMAI: 101 observaciones (serie 737233, base BIE-BISE); última May 26 = 101.629971; actualización BIE 23/07/2026 12:00:00 a. m..</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="62" t="inlineStr">
+        <is>
+          <t>• INEGI IMAI: 101 observaciones (serie 737234, base BIE-BISE); última May 26 = -0.007713; actualización BIE 23/07/2026 12:00:00 a. m..</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="62" t="inlineStr">
+        <is>
+          <t>• INEGI DESOCUP: 102 observaciones (serie 444603, base BIE-BISE); última Jun 26 = 0.028985; actualización BIE 24/07/2026 12:00:00 a. m..</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="62" t="inlineStr">
+        <is>
+          <t>• INEGI INPC: 102 observaciones (serie 334360, base BIE-BISE); última Jun 26 = 3.365977; actualización BIE 10/07/2026 12:00:00 a. m..</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="62" t="inlineStr">
+        <is>
+          <t>• INEGI INPC: 102 observaciones (serie 334452, base BIE-BISE); última Jun 26 = 4.03192; actualización BIE 10/07/2026 12:00:00 a. m..</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="62" t="inlineStr">
+        <is>
+          <t>• INEGI BALANZA: 102 observaciones (serie 33223, base BIE-BISE); última Jun 26 = 72551.015; actualización BIE 27/07/2026 12:00:00 a. m..</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="62" t="inlineStr">
+        <is>
+          <t>• INEGI BALANZA: 102 observaciones (serie 33226, base BIE-BISE); última Jun 26 = 68461.119; actualización BIE 27/07/2026 12:00:00 a. m..</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="62" t="inlineStr">
+        <is>
+          <t>• [IMFBCF] sin observaciones (estado: pendiente de confirmar serie).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="62" t="inlineStr">
+        <is>
+          <t>• [IOAE] sin observaciones (estado: pendiente de confirmar serie).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="62" t="inlineStr">
+        <is>
+          <t>• [EMIM] sin observaciones (estado: pendiente de confirmar serie).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="62" t="inlineStr">
+        <is>
+          <t>• [TIPOCAMBIO] sin observaciones (estado: pendiente de token).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="62" t="inlineStr">
+        <is>
+          <t>• [TASA] sin observaciones (estado: pendiente de token).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="62" t="inlineStr">
         <is>
           <t>• [RESERVAS] sin observaciones (estado: pendiente de token).</t>
         </is>

</xml_diff>